<commit_message>
add products table and ordernumber field, update screenshots and readme
</commit_message>
<xml_diff>
--- a/normalized_table.xlsx
+++ b/normalized_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anastasiia.kuzmina/Desktop/goit-rdb-hw-02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{42C9B2CB-E43D-C840-AF47-D33820C9F2A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2635E3-4606-6C41-975E-E4872C2C76F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4000" yWindow="2060" windowWidth="28040" windowHeight="17180" activeTab="2" xr2:uid="{34365902-6EB8-6449-8CCE-683D82C93CE0}"/>
+    <workbookView xWindow="19140" yWindow="2060" windowWidth="12900" windowHeight="17180" activeTab="2" xr2:uid="{34365902-6EB8-6449-8CCE-683D82C93CE0}"/>
   </bookViews>
   <sheets>
     <sheet name="1НФ" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="26">
   <si>
     <t>Таблицю нормалізовано до 1НФ</t>
   </si>
@@ -113,6 +113,12 @@
   </si>
   <si>
     <t>order_detail_id</t>
+  </si>
+  <si>
+    <t>Таблиця Товари</t>
+  </si>
+  <si>
+    <t>product_id</t>
   </si>
 </sst>
 </file>
@@ -175,23 +181,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <b val="0"/>
@@ -251,6 +252,40 @@
         <horizontal/>
       </border>
     </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="7"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -310,7 +345,7 @@
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{C8C9CF2B-4156-AF4B-90E7-B245AFC0CC44}" name="order_detail_id"/>
     <tableColumn id="2" xr3:uid="{74AB5A32-7ED6-E94E-B9AB-A92AC1E6ABDB}" name="order_id"/>
-    <tableColumn id="3" xr3:uid="{7DFE91EE-58E9-F842-BDC7-81D66069F333}" name="product_name" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{7DFE91EE-58E9-F842-BDC7-81D66069F333}" name="product_id" dataDxfId="5"/>
     <tableColumn id="4" xr3:uid="{EF764048-AD69-7C46-B651-A6D458FE4F62}" name="quantity"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -335,7 +370,18 @@
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{E8757DF7-9419-ED40-98DD-B210B2CAC19F}" name="order_id"/>
     <tableColumn id="2" xr3:uid="{6C9403BF-9511-C340-AD53-7500E1AC6ECD}" name="client_id"/>
-    <tableColumn id="3" xr3:uid="{2CCDC996-20AC-214A-9346-C9BEE4E68666}" name="order_date" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{2CCDC996-20AC-214A-9346-C9BEE4E68666}" name="order_date" dataDxfId="4"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D9E373A4-9217-534D-A12D-6489F5981392}" name="Table7" displayName="Table7" ref="A17:B20" totalsRowShown="0">
+  <autoFilter ref="A17:B20" xr:uid="{D9E373A4-9217-534D-A12D-6489F5981392}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{AB6B6153-5FBF-6747-B35B-69C2A147CEAF}" name="product_id"/>
+    <tableColumn id="2" xr3:uid="{DD66D7F7-8136-B545-BCE6-E18B1B1F97F8}" name="product_name" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -932,11 +978,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6881CF81-DF07-284E-84E1-022C4F6D1941}">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
-    <col min="2" max="2" width="13.5" customWidth="1"/>
+    <col min="2" max="2" width="15.1640625" customWidth="1"/>
     <col min="3" max="3" width="15.33203125" customWidth="1"/>
     <col min="7" max="7" width="12.33203125" customWidth="1"/>
   </cols>
@@ -1047,7 +1093,7 @@
         <v>2</v>
       </c>
       <c r="C10" t="s">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
         <v>4</v>
@@ -1060,8 +1106,8 @@
       <c r="B11">
         <v>101</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>8</v>
+      <c r="C11" s="2">
+        <v>1</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -1074,8 +1120,8 @@
       <c r="B12">
         <v>101</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>9</v>
+      <c r="C12" s="2">
+        <v>2</v>
       </c>
       <c r="D12">
         <v>2</v>
@@ -1088,8 +1134,8 @@
       <c r="B13">
         <v>102</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>10</v>
+      <c r="C13" s="2">
+        <v>3</v>
       </c>
       <c r="D13">
         <v>1</v>
@@ -1102,19 +1148,57 @@
       <c r="B14">
         <v>103</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>9</v>
+      <c r="C14" s="3">
+        <v>2</v>
       </c>
       <c r="D14">
         <v>4</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>2</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>3</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
apply review feedback by adding products table and order_number and updating screenshots and readme
</commit_message>
<xml_diff>
--- a/normalized_table.xlsx
+++ b/normalized_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anastasiia.kuzmina/Desktop/goit-rdb-hw-02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC2635E3-4606-6C41-975E-E4872C2C76F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562DAA3D-86F2-4B49-9FF3-466F753AB7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19140" yWindow="2060" windowWidth="12900" windowHeight="17180" activeTab="2" xr2:uid="{34365902-6EB8-6449-8CCE-683D82C93CE0}"/>
+    <workbookView xWindow="13720" yWindow="2060" windowWidth="18320" windowHeight="17180" activeTab="2" xr2:uid="{34365902-6EB8-6449-8CCE-683D82C93CE0}"/>
   </bookViews>
   <sheets>
     <sheet name="1НФ" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="27">
   <si>
     <t>Таблицю нормалізовано до 1НФ</t>
   </si>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>product_id</t>
+  </si>
+  <si>
+    <t>order_number</t>
   </si>
 </sst>
 </file>
@@ -181,18 +184,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="6">
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -256,9 +261,6 @@
       <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -307,7 +309,7 @@
     <tableColumn id="2" xr3:uid="{132202E0-2037-264A-90ED-31D6DF5B3218}" name="product_name"/>
     <tableColumn id="3" xr3:uid="{3E925124-D3EE-E846-A029-B3473708F583}" name="quantity"/>
     <tableColumn id="4" xr3:uid="{C9CD5D1C-4D9D-B14B-B8DD-88366FE5A3A2}" name="client_address"/>
-    <tableColumn id="5" xr3:uid="{48F6659B-171C-FF4F-B271-FC0573BFE50D}" name="order_date" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{48F6659B-171C-FF4F-B271-FC0573BFE50D}" name="order_date" dataDxfId="2"/>
     <tableColumn id="6" xr3:uid="{CBD49989-42D7-D44C-93EA-B65F3E50B912}" name="client_name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -319,7 +321,7 @@
   <autoFilter ref="A10:C14" xr:uid="{DAC681BD-23C0-2142-8EE6-B993615038F3}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{9E9094BA-3067-8E4F-8D80-2727CC2C0506}" name="order_id"/>
-    <tableColumn id="2" xr3:uid="{6D9CE018-B00E-5B49-B3EC-D4353288CFD8}" name="product_name" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{6D9CE018-B00E-5B49-B3EC-D4353288CFD8}" name="product_name" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{5290902D-4ABB-EA4D-B42C-9584511BD504}" name="quantity"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -333,7 +335,7 @@
     <tableColumn id="1" xr3:uid="{83792F05-952A-824B-A7BB-5C2E2B763262}" name="order_id"/>
     <tableColumn id="2" xr3:uid="{4DE3C343-A77F-0C41-A33E-19297940DC35}" name="client_name"/>
     <tableColumn id="3" xr3:uid="{B286C00A-FCAC-3A4D-9808-FE2B420FBA25}" name="client_address"/>
-    <tableColumn id="4" xr3:uid="{DFC2566D-D94F-5746-80BC-9F846EB7CFC1}" name="order_date" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{DFC2566D-D94F-5746-80BC-9F846EB7CFC1}" name="order_date" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -365,12 +367,13 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C9167A13-0CAA-1A41-BC21-15536DECC300}" name="Table6" displayName="Table6" ref="E4:G7" totalsRowShown="0">
-  <autoFilter ref="E4:G7" xr:uid="{C9167A13-0CAA-1A41-BC21-15536DECC300}"/>
-  <tableColumns count="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{C9167A13-0CAA-1A41-BC21-15536DECC300}" name="Table6" displayName="Table6" ref="E4:H7" totalsRowShown="0">
+  <autoFilter ref="E4:H7" xr:uid="{C9167A13-0CAA-1A41-BC21-15536DECC300}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{E8757DF7-9419-ED40-98DD-B210B2CAC19F}" name="order_id"/>
     <tableColumn id="2" xr3:uid="{6C9403BF-9511-C340-AD53-7500E1AC6ECD}" name="client_id"/>
     <tableColumn id="3" xr3:uid="{2CCDC996-20AC-214A-9346-C9BEE4E68666}" name="order_date" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{CC7D75BB-FE2C-7046-B058-570C0255ACB6}" name="order_number"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -381,7 +384,7 @@
   <autoFilter ref="A17:B20" xr:uid="{D9E373A4-9217-534D-A12D-6489F5981392}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{AB6B6153-5FBF-6747-B35B-69C2A147CEAF}" name="product_id"/>
-    <tableColumn id="2" xr3:uid="{DD66D7F7-8136-B545-BCE6-E18B1B1F97F8}" name="product_name" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{DD66D7F7-8136-B545-BCE6-E18B1B1F97F8}" name="product_name" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -978,7 +981,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6881CF81-DF07-284E-84E1-022C4F6D1941}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
@@ -987,12 +990,12 @@
     <col min="7" max="7" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1000,7 +1003,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1019,8 +1022,11 @@
       <c r="G4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1039,8 +1045,11 @@
       <c r="G5" s="1">
         <v>45000</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1059,8 +1068,11 @@
       <c r="G6" s="1">
         <v>45001</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>3</v>
       </c>
@@ -1079,13 +1091,16 @@
       <c r="G7" s="1">
         <v>45002</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1099,7 +1114,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>1</v>
       </c>
@@ -1113,7 +1128,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1127,7 +1142,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>3</v>
       </c>
@@ -1141,7 +1156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>4</v>
       </c>
@@ -1155,7 +1170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1172,7 +1187,7 @@
       <c r="A18">
         <v>1</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1180,7 +1195,7 @@
       <c r="A19">
         <v>2</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1188,7 +1203,7 @@
       <c r="A20">
         <v>3</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
sync order ids in 3NF table with db schema
</commit_message>
<xml_diff>
--- a/normalized_table.xlsx
+++ b/normalized_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anastasiia.kuzmina/Desktop/goit-rdb-hw-02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562DAA3D-86F2-4B49-9FF3-466F753AB7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09071105-A471-7C45-974B-8A296676038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13720" yWindow="2060" windowWidth="18320" windowHeight="17180" activeTab="2" xr2:uid="{34365902-6EB8-6449-8CCE-683D82C93CE0}"/>
   </bookViews>
@@ -371,9 +371,9 @@
   <autoFilter ref="E4:H7" xr:uid="{C9167A13-0CAA-1A41-BC21-15536DECC300}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{E8757DF7-9419-ED40-98DD-B210B2CAC19F}" name="order_id"/>
+    <tableColumn id="5" xr3:uid="{417EC2B1-B9A2-CD4C-8F4F-6E24CA6FBB88}" name="order_number"/>
     <tableColumn id="2" xr3:uid="{6C9403BF-9511-C340-AD53-7500E1AC6ECD}" name="client_id"/>
     <tableColumn id="3" xr3:uid="{2CCDC996-20AC-214A-9346-C9BEE4E68666}" name="order_date" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{CC7D75BB-FE2C-7046-B058-570C0255ACB6}" name="order_number"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight12" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -988,6 +988,7 @@
     <col min="2" max="2" width="15.1640625" customWidth="1"/>
     <col min="3" max="3" width="15.33203125" customWidth="1"/>
     <col min="7" max="7" width="12.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
@@ -1017,13 +1018,13 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="s">
         <v>22</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>6</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1037,16 +1038,16 @@
         <v>11</v>
       </c>
       <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
         <v>101</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>1</v>
       </c>
-      <c r="G5" s="1">
+      <c r="H5" s="1">
         <v>45000</v>
-      </c>
-      <c r="H5">
-        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1060,16 +1061,16 @@
         <v>12</v>
       </c>
       <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
         <v>102</v>
       </c>
-      <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6" s="1">
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6" s="1">
         <v>45001</v>
-      </c>
-      <c r="H6">
-        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1083,16 +1084,16 @@
         <v>13</v>
       </c>
       <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
         <v>103</v>
       </c>
-      <c r="F7">
+      <c r="G7">
         <v>3</v>
       </c>
-      <c r="G7" s="1">
+      <c r="H7" s="1">
         <v>45002</v>
-      </c>
-      <c r="H7">
-        <v>103</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1130,7 +1131,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B12">
         <v>101</v>
@@ -1144,7 +1145,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B13">
         <v>102</v>
@@ -1158,7 +1159,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B14">
         <v>103</v>

</xml_diff>

<commit_message>
fix order_detail_id and order_id in 3NF order details table
</commit_message>
<xml_diff>
--- a/normalized_table.xlsx
+++ b/normalized_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anastasiia.kuzmina/Desktop/goit-rdb-hw-02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09071105-A471-7C45-974B-8A296676038E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AB1E865-B88C-F045-A6F9-15933498C6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="13720" yWindow="2060" windowWidth="18320" windowHeight="17180" activeTab="2" xr2:uid="{34365902-6EB8-6449-8CCE-683D82C93CE0}"/>
   </bookViews>
@@ -987,6 +987,7 @@
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="15.1640625" customWidth="1"/>
     <col min="3" max="3" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="16.1640625" customWidth="1"/>
     <col min="7" max="7" width="12.33203125" customWidth="1"/>
     <col min="8" max="8" width="12.1640625" customWidth="1"/>
   </cols>
@@ -1120,7 +1121,7 @@
         <v>1</v>
       </c>
       <c r="B11">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2">
         <v>1</v>
@@ -1131,10 +1132,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12">
         <v>1</v>
-      </c>
-      <c r="B12">
-        <v>101</v>
       </c>
       <c r="C12" s="2">
         <v>2</v>
@@ -1145,10 +1146,10 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B13">
-        <v>102</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2">
         <v>3</v>
@@ -1159,10 +1160,10 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14">
+        <v>4</v>
+      </c>
+      <c r="B14">
         <v>3</v>
-      </c>
-      <c r="B14">
-        <v>103</v>
       </c>
       <c r="C14" s="3">
         <v>2</v>

</xml_diff>